<commit_message>
added in another system
</commit_message>
<xml_diff>
--- a/server/Configuration_Output.xlsx
+++ b/server/Configuration_Output.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20357"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meena\Downloads\New folder\server\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://exlservicenam-my.sharepoint.com/personal/utkarsh258376_exlservice_com/Documents/Documents/fraud-signal-studio/server/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9C5E23-1EF8-4EB6-A489-DDCCB19AED64}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_F54B613CDC488CC9A7A6BAAD6474A936C82B56E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1573D52-10D6-4CC8-88D3-E817E4C68A39}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19008" windowHeight="7500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dim_MarkerScoringConfig" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1472" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1485" uniqueCount="120">
   <si>
     <t>ScenarioID</t>
   </si>
@@ -258,28 +258,46 @@
     <t>FabricTechnicalSpec</t>
   </si>
   <si>
+    <t>REQ-006</t>
+  </si>
+  <si>
+    <t>hello</t>
+  </si>
+  <si>
+    <t>Policy Issuance/Application</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Flag</t>
+  </si>
+  <si>
+    <t>utkarsh gaur</t>
+  </si>
+  <si>
+    <t>Utkarsh.Gaur@exlservice.com</t>
+  </si>
+  <si>
+    <t>Pending Review</t>
+  </si>
+  <si>
+    <t>2026-05-28T08:06:44.938Z</t>
+  </si>
+  <si>
     <t>REQ-005</t>
   </si>
   <si>
     <t>signal</t>
   </si>
   <si>
-    <t>Policy Issuance/Application</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Flag</t>
-  </si>
-  <si>
     <t>utkarsh</t>
   </si>
   <si>
     <t>utkarsh@gmail.com</t>
   </si>
   <si>
-    <t>Pending Review</t>
+    <t>Under Review</t>
   </si>
   <si>
     <t>2026-05-28T05:36:13.150Z</t>
@@ -327,12 +345,6 @@
     <t>agent selling in different region</t>
   </si>
   <si>
-    <t>utkarsh gaur</t>
-  </si>
-  <si>
-    <t>Utkarsh.Gaur@exlservice.com</t>
-  </si>
-  <si>
     <t>2026-05-27T07:14:15.786Z</t>
   </si>
   <si>
@@ -366,24 +378,21 @@
     <t>jane.doe@company.com</t>
   </si>
   <si>
-    <t>Under Review</t>
-  </si>
-  <si>
     <t>2026-05-25T10:00:00Z</t>
   </si>
   <si>
-    <t xml:space="preserve">### Microsoft Fabric Data Agent Technical Specification_x000D_
-_x000D_
-#### 1. Recommended Data Mapping_x000D_
-* **Primary Target Table**: `factpartynamedata`_x000D_
-_x000D_
-#### 2. SQL Implementation (Lakehouse Query)_x000D_
-```sql_x000D_
-SELECT pb.PolicyID, pb.BeneficiaryID, pb.ChangeDate_x000D_
-FROM factpartynamedata pb_x000D_
-JOIN factpolicycontractdata p ON pb.PolicyID = p.PolicyID_x000D_
-WHERE DATEDIFF(day, p.IssueDate, pb.ChangeDate) &lt;= 30;_x000D_
-```_x000D_
+    <t xml:space="preserve">### Microsoft Fabric Data Agent Technical Specification_x000D__x000D_
+_x000D__x000D_
+#### 1. Recommended Data Mapping_x000D__x000D_
+* **Primary Target Table**: `factpartynamedata`_x000D__x000D_
+_x000D__x000D_
+#### 2. SQL Implementation (Lakehouse Query)_x000D__x000D_
+```sql_x000D__x000D_
+SELECT pb.PolicyID, pb.BeneficiaryID, pb.ChangeDate_x000D__x000D_
+FROM factpartynamedata pb_x000D__x000D_
+JOIN factpolicycontractdata p ON pb.PolicyID = p.PolicyID_x000D__x000D_
+WHERE DATEDIFF(day, p.IssueDate, pb.ChangeDate) &lt;= 30;_x000D__x000D_
+```_x000D__x000D_
 </t>
   </si>
 </sst>
@@ -421,7 +430,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -762,9 +771,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J274"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -796,7 +805,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -828,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -860,7 +869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -892,7 +901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -924,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -956,7 +965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -988,7 +997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1020,7 +1029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1052,7 +1061,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1084,7 +1093,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1116,7 +1125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1148,7 +1157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1180,7 +1189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1212,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1244,7 +1253,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -1276,7 +1285,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -1308,7 +1317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1340,7 +1349,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1372,7 +1381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -1404,7 +1413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -1436,7 +1445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -1468,7 +1477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1500,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -1532,7 +1541,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -1564,7 +1573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -1596,7 +1605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -1628,7 +1637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -1660,7 +1669,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -1692,7 +1701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>10</v>
       </c>
@@ -1724,7 +1733,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -1756,7 +1765,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1788,7 +1797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -1820,7 +1829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -1852,7 +1861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -1884,7 +1893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>10</v>
       </c>
@@ -1916,7 +1925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>10</v>
       </c>
@@ -1948,7 +1957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -1980,7 +1989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>10</v>
       </c>
@@ -2012,7 +2021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>10</v>
       </c>
@@ -2044,7 +2053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>10</v>
       </c>
@@ -2076,7 +2085,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>10</v>
       </c>
@@ -2108,7 +2117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -2140,7 +2149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>10</v>
       </c>
@@ -2172,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>10</v>
       </c>
@@ -2204,7 +2213,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>10</v>
       </c>
@@ -2236,7 +2245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>10</v>
       </c>
@@ -2268,7 +2277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>10</v>
       </c>
@@ -2300,7 +2309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>10</v>
       </c>
@@ -2332,7 +2341,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>10</v>
       </c>
@@ -2364,7 +2373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>10</v>
       </c>
@@ -2396,7 +2405,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>10</v>
       </c>
@@ -2428,7 +2437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>10</v>
       </c>
@@ -2460,7 +2469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>10</v>
       </c>
@@ -2492,7 +2501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>10</v>
       </c>
@@ -2524,7 +2533,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>10</v>
       </c>
@@ -2556,7 +2565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>10</v>
       </c>
@@ -2588,7 +2597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>10</v>
       </c>
@@ -2620,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>10</v>
       </c>
@@ -2652,7 +2661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>10</v>
       </c>
@@ -2684,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>10</v>
       </c>
@@ -2716,7 +2725,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>10</v>
       </c>
@@ -2748,7 +2757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>10</v>
       </c>
@@ -2780,7 +2789,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>10</v>
       </c>
@@ -2812,7 +2821,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -2844,7 +2853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>10</v>
       </c>
@@ -2876,7 +2885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>10</v>
       </c>
@@ -2908,7 +2917,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>10</v>
       </c>
@@ -2940,7 +2949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>10</v>
       </c>
@@ -2972,7 +2981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>10</v>
       </c>
@@ -3004,7 +3013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>10</v>
       </c>
@@ -3036,7 +3045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>10</v>
       </c>
@@ -3068,7 +3077,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>10</v>
       </c>
@@ -3100,7 +3109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>10</v>
       </c>
@@ -3132,7 +3141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>10</v>
       </c>
@@ -3164,7 +3173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>10</v>
       </c>
@@ -3196,7 +3205,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>10</v>
       </c>
@@ -3228,7 +3237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>10</v>
       </c>
@@ -3260,7 +3269,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>10</v>
       </c>
@@ -3292,7 +3301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>10</v>
       </c>
@@ -3324,7 +3333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>10</v>
       </c>
@@ -3356,7 +3365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>10</v>
       </c>
@@ -3388,7 +3397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>10</v>
       </c>
@@ -3420,7 +3429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>10</v>
       </c>
@@ -3452,7 +3461,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>10</v>
       </c>
@@ -3484,7 +3493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>10</v>
       </c>
@@ -3516,7 +3525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>10</v>
       </c>
@@ -3548,7 +3557,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>10</v>
       </c>
@@ -3580,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>10</v>
       </c>
@@ -3612,7 +3621,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>10</v>
       </c>
@@ -3644,7 +3653,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>10</v>
       </c>
@@ -3676,7 +3685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>10</v>
       </c>
@@ -3708,7 +3717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>53</v>
       </c>
@@ -3740,7 +3749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>53</v>
       </c>
@@ -3772,7 +3781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>53</v>
       </c>
@@ -3804,7 +3813,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>53</v>
       </c>
@@ -3836,7 +3845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>53</v>
       </c>
@@ -3868,7 +3877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>53</v>
       </c>
@@ -3900,7 +3909,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>53</v>
       </c>
@@ -3932,7 +3941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>53</v>
       </c>
@@ -3964,7 +3973,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>53</v>
       </c>
@@ -3996,7 +4005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>53</v>
       </c>
@@ -4028,7 +4037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>53</v>
       </c>
@@ -4060,7 +4069,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>53</v>
       </c>
@@ -4092,7 +4101,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>53</v>
       </c>
@@ -4124,7 +4133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>53</v>
       </c>
@@ -4156,7 +4165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>53</v>
       </c>
@@ -4188,7 +4197,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>53</v>
       </c>
@@ -4220,7 +4229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>53</v>
       </c>
@@ -4252,7 +4261,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>53</v>
       </c>
@@ -4284,7 +4293,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>53</v>
       </c>
@@ -4316,7 +4325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>53</v>
       </c>
@@ -4348,7 +4357,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>53</v>
       </c>
@@ -4380,7 +4389,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>53</v>
       </c>
@@ -4412,7 +4421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>53</v>
       </c>
@@ -4444,7 +4453,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>53</v>
       </c>
@@ -4476,7 +4485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>53</v>
       </c>
@@ -4508,7 +4517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>53</v>
       </c>
@@ -4540,7 +4549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>53</v>
       </c>
@@ -4572,7 +4581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>53</v>
       </c>
@@ -4604,7 +4613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>53</v>
       </c>
@@ -4636,7 +4645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>53</v>
       </c>
@@ -4668,7 +4677,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>53</v>
       </c>
@@ -4700,7 +4709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>53</v>
       </c>
@@ -4732,7 +4741,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>53</v>
       </c>
@@ -4764,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>53</v>
       </c>
@@ -4796,7 +4805,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>53</v>
       </c>
@@ -4828,7 +4837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>53</v>
       </c>
@@ -4860,7 +4869,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>53</v>
       </c>
@@ -4892,7 +4901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>53</v>
       </c>
@@ -4924,7 +4933,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>53</v>
       </c>
@@ -4956,7 +4965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>53</v>
       </c>
@@ -4988,7 +4997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>53</v>
       </c>
@@ -5020,7 +5029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>53</v>
       </c>
@@ -5052,7 +5061,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>53</v>
       </c>
@@ -5084,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>53</v>
       </c>
@@ -5116,7 +5125,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>53</v>
       </c>
@@ -5148,7 +5157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>53</v>
       </c>
@@ -5180,7 +5189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>53</v>
       </c>
@@ -5212,7 +5221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>53</v>
       </c>
@@ -5244,7 +5253,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>53</v>
       </c>
@@ -5276,7 +5285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>53</v>
       </c>
@@ -5308,7 +5317,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>53</v>
       </c>
@@ -5340,7 +5349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>53</v>
       </c>
@@ -5372,7 +5381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>53</v>
       </c>
@@ -5404,7 +5413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>53</v>
       </c>
@@ -5436,7 +5445,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>53</v>
       </c>
@@ -5468,7 +5477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>53</v>
       </c>
@@ -5500,7 +5509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>53</v>
       </c>
@@ -5532,7 +5541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>53</v>
       </c>
@@ -5564,7 +5573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>53</v>
       </c>
@@ -5596,7 +5605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>53</v>
       </c>
@@ -5628,7 +5637,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>53</v>
       </c>
@@ -5660,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>53</v>
       </c>
@@ -5692,7 +5701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>53</v>
       </c>
@@ -5724,7 +5733,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>53</v>
       </c>
@@ -5756,7 +5765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>53</v>
       </c>
@@ -5788,7 +5797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>53</v>
       </c>
@@ -5820,7 +5829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>53</v>
       </c>
@@ -5852,7 +5861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>53</v>
       </c>
@@ -5884,7 +5893,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>53</v>
       </c>
@@ -5916,7 +5925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>53</v>
       </c>
@@ -5948,7 +5957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>53</v>
       </c>
@@ -5980,7 +5989,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>53</v>
       </c>
@@ -6012,7 +6021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>53</v>
       </c>
@@ -6044,7 +6053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>53</v>
       </c>
@@ -6076,7 +6085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>53</v>
       </c>
@@ -6108,7 +6117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>53</v>
       </c>
@@ -6140,7 +6149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>53</v>
       </c>
@@ -6172,7 +6181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>53</v>
       </c>
@@ -6204,7 +6213,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>53</v>
       </c>
@@ -6236,7 +6245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>53</v>
       </c>
@@ -6268,7 +6277,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>53</v>
       </c>
@@ -6300,7 +6309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>53</v>
       </c>
@@ -6332,7 +6341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>53</v>
       </c>
@@ -6364,7 +6373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>53</v>
       </c>
@@ -6396,7 +6405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>53</v>
       </c>
@@ -6428,7 +6437,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>53</v>
       </c>
@@ -6460,7 +6469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>53</v>
       </c>
@@ -6492,7 +6501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>53</v>
       </c>
@@ -6524,7 +6533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>53</v>
       </c>
@@ -6556,7 +6565,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>53</v>
       </c>
@@ -6588,7 +6597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>53</v>
       </c>
@@ -6620,7 +6629,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>55</v>
       </c>
@@ -6652,7 +6661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>55</v>
       </c>
@@ -6684,7 +6693,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>55</v>
       </c>
@@ -6716,7 +6725,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>55</v>
       </c>
@@ -6748,7 +6757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>55</v>
       </c>
@@ -6780,7 +6789,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>55</v>
       </c>
@@ -6812,7 +6821,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>55</v>
       </c>
@@ -6844,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>55</v>
       </c>
@@ -6876,7 +6885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>55</v>
       </c>
@@ -6908,7 +6917,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="193" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>55</v>
       </c>
@@ -6940,7 +6949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>55</v>
       </c>
@@ -6972,7 +6981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>55</v>
       </c>
@@ -7004,7 +7013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>55</v>
       </c>
@@ -7036,7 +7045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>55</v>
       </c>
@@ -7068,7 +7077,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>55</v>
       </c>
@@ -7100,7 +7109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="199" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>55</v>
       </c>
@@ -7132,7 +7141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>55</v>
       </c>
@@ -7164,7 +7173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>55</v>
       </c>
@@ -7196,7 +7205,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="202" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>55</v>
       </c>
@@ -7228,7 +7237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>55</v>
       </c>
@@ -7260,7 +7269,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>55</v>
       </c>
@@ -7292,7 +7301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="205" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>55</v>
       </c>
@@ -7324,7 +7333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>55</v>
       </c>
@@ -7356,7 +7365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>55</v>
       </c>
@@ -7388,7 +7397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>55</v>
       </c>
@@ -7420,7 +7429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>55</v>
       </c>
@@ -7452,7 +7461,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>55</v>
       </c>
@@ -7484,7 +7493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>55</v>
       </c>
@@ -7516,7 +7525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>55</v>
       </c>
@@ -7548,7 +7557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>55</v>
       </c>
@@ -7580,7 +7589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>55</v>
       </c>
@@ -7612,7 +7621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>55</v>
       </c>
@@ -7644,7 +7653,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="216" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>55</v>
       </c>
@@ -7676,7 +7685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>55</v>
       </c>
@@ -7708,7 +7717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="218" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>55</v>
       </c>
@@ -7740,7 +7749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>55</v>
       </c>
@@ -7772,7 +7781,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="220" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>55</v>
       </c>
@@ -7804,7 +7813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>55</v>
       </c>
@@ -7836,7 +7845,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="222" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>55</v>
       </c>
@@ -7868,7 +7877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>55</v>
       </c>
@@ -7900,7 +7909,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="224" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>55</v>
       </c>
@@ -7932,7 +7941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>55</v>
       </c>
@@ -7964,7 +7973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>55</v>
       </c>
@@ -7996,7 +8005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>55</v>
       </c>
@@ -8028,7 +8037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="228" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>55</v>
       </c>
@@ -8060,7 +8069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>55</v>
       </c>
@@ -8092,7 +8101,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="230" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>55</v>
       </c>
@@ -8124,7 +8133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>55</v>
       </c>
@@ -8156,7 +8165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="232" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>55</v>
       </c>
@@ -8188,7 +8197,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>55</v>
       </c>
@@ -8220,7 +8229,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="234" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>55</v>
       </c>
@@ -8252,7 +8261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>55</v>
       </c>
@@ -8284,7 +8293,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="236" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>55</v>
       </c>
@@ -8316,7 +8325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>55</v>
       </c>
@@ -8348,7 +8357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="238" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>55</v>
       </c>
@@ -8380,7 +8389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>55</v>
       </c>
@@ -8412,7 +8421,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="240" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>55</v>
       </c>
@@ -8444,7 +8453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>55</v>
       </c>
@@ -8476,7 +8485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="242" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>55</v>
       </c>
@@ -8508,7 +8517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>55</v>
       </c>
@@ -8540,7 +8549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>55</v>
       </c>
@@ -8572,7 +8581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>55</v>
       </c>
@@ -8604,7 +8613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>55</v>
       </c>
@@ -8636,7 +8645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="247" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>55</v>
       </c>
@@ -8668,7 +8677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>55</v>
       </c>
@@ -8700,7 +8709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="249" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>55</v>
       </c>
@@ -8732,7 +8741,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="250" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>55</v>
       </c>
@@ -8764,7 +8773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>55</v>
       </c>
@@ -8796,7 +8805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="252" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>55</v>
       </c>
@@ -8828,7 +8837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="253" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>55</v>
       </c>
@@ -8860,7 +8869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>55</v>
       </c>
@@ -8892,7 +8901,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>55</v>
       </c>
@@ -8924,7 +8933,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="256" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>55</v>
       </c>
@@ -8956,7 +8965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>55</v>
       </c>
@@ -8988,7 +8997,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="258" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>55</v>
       </c>
@@ -9020,7 +9029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="259" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>55</v>
       </c>
@@ -9052,7 +9061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>55</v>
       </c>
@@ -9084,7 +9093,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>55</v>
       </c>
@@ -9116,7 +9125,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="262" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>55</v>
       </c>
@@ -9148,7 +9157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>55</v>
       </c>
@@ -9180,7 +9189,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>55</v>
       </c>
@@ -9212,7 +9221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="265" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>55</v>
       </c>
@@ -9244,7 +9253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>55</v>
       </c>
@@ -9276,7 +9285,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="267" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>55</v>
       </c>
@@ -9308,7 +9317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>55</v>
       </c>
@@ -9340,7 +9349,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="269" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>55</v>
       </c>
@@ -9372,7 +9381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="270" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>55</v>
       </c>
@@ -9404,7 +9413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>55</v>
       </c>
@@ -9436,7 +9445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="272" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>55</v>
       </c>
@@ -9468,7 +9477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>55</v>
       </c>
@@ -9500,7 +9509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>55</v>
       </c>
@@ -9543,9 +9552,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9568,7 +9577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -9591,7 +9600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -9614,7 +9623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>55</v>
       </c>
@@ -9647,10 +9656,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>65</v>
       </c>
@@ -9691,7 +9700,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -9723,7 +9732,7 @@
         <v>84</v>
       </c>
       <c r="K2" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="L2" t="s">
         <v>86</v>
@@ -9732,7 +9741,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -9749,7 +9758,7 @@
         <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G3" t="s">
         <v>82</v>
@@ -9758,30 +9767,30 @@
         <v>81</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="K3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="L3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="M3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="D4" t="s">
         <v>81</v>
@@ -9790,7 +9799,7 @@
         <v>81</v>
       </c>
       <c r="F4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G4" t="s">
         <v>82</v>
@@ -9799,30 +9808,30 @@
         <v>81</v>
       </c>
       <c r="I4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="J4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L4" t="s">
         <v>95</v>
-      </c>
-      <c r="K4" t="s">
-        <v>96</v>
-      </c>
-      <c r="L4" t="s">
-        <v>97</v>
       </c>
       <c r="M4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" t="s">
         <v>98</v>
-      </c>
-      <c r="B5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C5" t="s">
-        <v>92</v>
       </c>
       <c r="D5" t="s">
         <v>81</v>
@@ -9831,7 +9840,7 @@
         <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G5" t="s">
         <v>82</v>
@@ -9840,13 +9849,13 @@
         <v>81</v>
       </c>
       <c r="I5" t="s">
+        <v>100</v>
+      </c>
+      <c r="J5" t="s">
         <v>101</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>102</v>
-      </c>
-      <c r="K5" t="s">
-        <v>85</v>
       </c>
       <c r="L5" t="s">
         <v>103</v>
@@ -9855,7 +9864,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>104</v>
       </c>
@@ -9863,43 +9872,84 @@
         <v>105</v>
       </c>
       <c r="C6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" t="s">
         <v>106</v>
       </c>
-      <c r="D6" t="s">
+      <c r="G6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K6" t="s">
+        <v>85</v>
+      </c>
+      <c r="L6" t="s">
         <v>107</v>
       </c>
-      <c r="E6" t="s">
+      <c r="M6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>108</v>
       </c>
-      <c r="F6" t="s">
+      <c r="B7" t="s">
         <v>109</v>
       </c>
-      <c r="G6" t="s">
+      <c r="C7" t="s">
         <v>110</v>
       </c>
-      <c r="H6" t="s">
+      <c r="D7" t="s">
         <v>111</v>
       </c>
-      <c r="I6" t="s">
+      <c r="E7" t="s">
         <v>112</v>
       </c>
-      <c r="J6" t="s">
+      <c r="F7" t="s">
         <v>113</v>
       </c>
-      <c r="K6" t="s">
+      <c r="G7" t="s">
         <v>114</v>
       </c>
-      <c r="L6" t="s">
+      <c r="H7" t="s">
         <v>115</v>
       </c>
-      <c r="M6" t="s">
+      <c r="I7" t="s">
         <v>116</v>
+      </c>
+      <c r="J7" t="s">
+        <v>117</v>
+      </c>
+      <c r="K7" t="s">
+        <v>91</v>
+      </c>
+      <c r="L7" t="s">
+        <v>118</v>
+      </c>
+      <c r="M7" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:M1 A3:M6 A2:J2 L2:M2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:M1 A3:M7 A2:J2 L2:M2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>